<commit_message>
finalize demo and update logic
</commit_message>
<xml_diff>
--- a/output/discrepancy_report_Demo Campaign.xlsx
+++ b/output/discrepancy_report_Demo Campaign.xlsx
@@ -476,29 +476,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1465</t>
+          <t>491I</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>象鼻芝士肠肉酱大热狗</t>
+          <t>独享热狗小吃3件套</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>18.9</v>
+        <v>26.9</v>
       </c>
       <c r="F2" t="n">
-        <v>18.9</v>
+        <v>26.9</v>
       </c>
       <c r="G2" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="H2" t="n">
-        <v>16</v>
-      </c>
+        <v>24.9</v>
+      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
-          <t>尝新价不一致</t>
+          <t>缺少实际尝新价</t>
         </is>
       </c>
     </row>
@@ -515,29 +513,25 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>491I</t>
+          <t>492I</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>独享热狗小吃3件套</t>
+          <t>买人气比萨送象鼻芝士肠肉酱大热狗</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>26.9</v>
+        <v>42.9</v>
       </c>
       <c r="F3" t="n">
-        <v>26.9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>24.9</v>
-      </c>
-      <c r="H3" t="n">
-        <v>40</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>尝新价不一致</t>
+          <t>活动价不一致</t>
         </is>
       </c>
     </row>
@@ -549,30 +543,34 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>美团外卖</t>
+          <t>饿了么</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>495I</t>
+          <t>1465</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>欢聚下午茶热狗小吃5件套</t>
+          <t>象鼻芝士肠肉酱大热狗</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>39.9</v>
+        <v>18.9</v>
       </c>
       <c r="F4" t="n">
-        <v>36.9</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+        <v>18.9</v>
+      </c>
+      <c r="G4" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="H4" t="n">
+        <v>16</v>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>活动价不一致</t>
+          <t>尝新价不一致</t>
         </is>
       </c>
     </row>

</xml_diff>